<commit_message>
feat: adjust load buttons when zero projects, add portfolio directory management, and add IT - InfoSec sample xls
- When zero projects, load buttons say 'Load Projects' without hardcoded counts and count badges are hidden
- Add portfolio creation and deletion management in store and Lifecycle UI
- Add IT - InfoSec portfolio and sample projects in .xls and .xlsx formats under data/ and data/portfolios/

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/portfolios/portfolio_all_100_projects.xlsx
+++ b/data/portfolios/portfolio_all_100_projects.xlsx
@@ -689,7 +689,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -1547,7 +1547,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -1690,7 +1690,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1837,7 +1837,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -1976,7 +1976,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -2401,7 +2401,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -2687,7 +2687,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -2834,7 +2834,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -2981,7 +2981,7 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -3124,7 +3124,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -3406,7 +3406,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -3549,7 +3549,7 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -3696,7 +3696,7 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -3835,7 +3835,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -4260,7 +4260,7 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -4546,7 +4546,7 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -4689,7 +4689,7 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -4832,7 +4832,7 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -4971,7 +4971,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -5110,7 +5110,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -5249,7 +5249,7 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -5388,7 +5388,7 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -5527,7 +5527,7 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -5670,7 +5670,7 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -5813,7 +5813,7 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -5952,7 +5952,7 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -6091,7 +6091,7 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -6230,7 +6230,7 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>IT InfoSec</t>
+          <t>IT - InfoSec</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">

</xml_diff>